<commit_message>
forest land new format
</commit_message>
<xml_diff>
--- a/uploads/excels/Private_Land_Format_(1)_(1).xlsx
+++ b/uploads/excels/Private_Land_Format_(1)_(1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maasuser\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65248E01-EA17-4E5D-86DF-9F3B56179C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{266550B4-84F4-4C77-AF28-359F744CCF00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="230">
   <si>
     <t>SES Survey No.</t>
   </si>
@@ -1702,16 +1702,16 @@
         <v>2</v>
       </c>
       <c r="BF2" s="5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH2" s="5">
         <v>1</v>
       </c>
-      <c r="BI2" s="5" t="s">
-        <v>93</v>
+      <c r="BI2" s="5">
+        <v>1</v>
       </c>
       <c r="BJ2" s="7" t="s">
         <v>70</v>

</xml_diff>